<commit_message>
Updated version of Excel sheet Model
Updated version of Excel sheet Model with all 3 figures as well as MC label added.
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasmindeguzman/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasmindeguzman/Library/Mobile Documents/com~apple~CloudDocs/1 UH MBA/620 Micro and Macro Economoics/GitHub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBF9695-0E21-9F44-93CA-6D681CA3393F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BAEA7254-428F-8D4D-A510-441B9C1B62EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32440" yWindow="-5440" windowWidth="29260" windowHeight="19900" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5040" yWindow="660" windowWidth="23140" windowHeight="18460" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -962,6 +962,64 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="rnd">
+                      <a:solidFill>
+                        <a:schemeClr val="dk1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:xVal>
             <c:numRef>
               <c:f>'Marginal-Cost Schedules'!$J$7:$J$8</c:f>
@@ -1672,6 +1730,64 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="rnd">
+                      <a:solidFill>
+                        <a:schemeClr val="dk1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:xVal>
             <c:numRef>
               <c:f>'Marginal-Cost Schedules'!$J$31:$J$32</c:f>
@@ -2253,6 +2369,834 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="20" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" b="1"/>
+              <a:t>Mesclun Marginal Cost vs. Market Price</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="20" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Mesclun Price</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:alpha val="70000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:prstDash val="sysDot"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:gradFill>
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent1">
+                      <a:tint val="50000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="35000">
+                    <a:schemeClr val="accent1">
+                      <a:tint val="37000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent1">
+                      <a:tint val="15000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="16200000" scaled="1"/>
+                <a:tileRect/>
+              </a:gradFill>
+              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:shade val="95000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="rnd">
+                      <a:solidFill>
+                        <a:schemeClr val="dk1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Marginal-Cost Schedules'!$J$56:$J$57</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>30</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Marginal-Cost Schedules'!$K$56:$K$57</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2700</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FD7A-434C-BFF6-12CA2F633672}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Marginal Cost</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:alpha val="70000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:prstDash val="sysDot"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:gradFill>
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent2">
+                      <a:tint val="50000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="35000">
+                    <a:schemeClr val="accent2">
+                      <a:tint val="37000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent2">
+                      <a:tint val="15000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="16200000" scaled="1"/>
+                <a:tileRect/>
+              </a:gradFill>
+              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:shade val="95000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Marginal-Cost Schedules'!$A$56:$A$86</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>30</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Marginal-Cost Schedules'!$H$56:$H$86</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0.00</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="1">
+                  <c:v>2462.03125</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2501.58203125</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2541.8743896484366</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2582.920684814454</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2624.7334694862348</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2667.3254924178127</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2710.7097013180683</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2754.8992458326466</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2799.9074805692508</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2845.7479681671139</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2892.4344824110776</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2939.9810113911262</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2988.4017607077876</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2522.5810943551696</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1983.9619249331008</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2009.5273589841818</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2035.5594348357699</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2062.0658239338081</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2089.0543165975978</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2116.532823793008</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2144.5093789313105</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2172.9921396943828</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2201.9893898860464</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2231.5095413106901</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2261.5611356787776</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2292.1528465402444</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2323.2934812457679</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2354.9919829366991</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2387.2574325634341</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2420.0990509335097</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-FD7A-434C-BFF6-12CA2F633672}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="172224767"/>
+        <c:axId val="170598719"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="172224767"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Mesclun Beds</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="rnd">
+            <a:solidFill>
+              <a:schemeClr val="dk1">
+                <a:lumMod val="20000"/>
+                <a:lumOff val="80000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="170598719"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="170598719"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" b="1"/>
+                  <a:t>Marginal Cost ($)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="rnd">
+            <a:solidFill>
+              <a:schemeClr val="dk1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="172224767"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="lt1">
+                <a:alpha val="0"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="lt1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -2294,6 +3238,46 @@
 </file>
 
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -3435,20 +4419,571 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="246">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="2">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="1"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:shade val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="2">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="1"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:shade val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="2"/>
+    <cs:effectRef idx="1"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:alpha val="70000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="2">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="1"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:shade val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200" spc="0" baseline="0"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill>
+        <a:gsLst>
+          <a:gs pos="100000">
+            <a:schemeClr val="lt1">
+              <a:lumMod val="95000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="0">
+            <a:schemeClr val="lt1">
+              <a:alpha val="0"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:lin ang="5400000" scaled="0"/>
+      </a:gradFill>
+    </cs:spPr>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="50000"/>
+        <a:lumOff val="50000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" kern="1200" cap="none" spc="20" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200" spc="0" baseline="0"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>158750</xdr:rowOff>
+      <xdr:colOff>577850</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>323850</xdr:colOff>
+      <xdr:colOff>527050</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>44450</xdr:rowOff>
+      <xdr:rowOff>107950</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3504,6 +5039,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>368300</xdr:colOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D1B72FEB-4235-8701-5C21-C2B908C88CD2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -5888,7 +7459,7 @@
         <v>1670.9013431626554</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="18">
         <v>18</v>
       </c>
@@ -5921,7 +7492,7 @@
         <v>1589.1387909931072</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" s="18">
         <v>19</v>
       </c>
@@ -5954,7 +7525,7 @@
         <v>1638.1753169880685</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="18">
         <v>20</v>
       </c>
@@ -5987,7 +7558,7 @@
         <v>1688.9454575384007</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" s="19" t="s">
         <v>101</v>
       </c>
@@ -6004,7 +7575,7 @@
       <c r="G52" s="29"/>
       <c r="H52" s="29"/>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" s="30" t="s">
         <v>104</v>
       </c>
@@ -6016,7 +7587,7 @@
       <c r="G54" s="30"/>
       <c r="H54" s="30"/>
     </row>
-    <row r="55" spans="1:8" ht="30" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" ht="30" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>93</v>
       </c>
@@ -6042,7 +7613,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" s="18">
         <v>0</v>
       </c>
@@ -6071,8 +7642,14 @@
         <v>0</v>
       </c>
       <c r="H56" s="18"/>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="J56">
+        <v>1</v>
+      </c>
+      <c r="K56">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" s="18">
         <v>1</v>
       </c>
@@ -6104,8 +7681,14 @@
         <f t="shared" ref="H57:H86" si="20">G57-G56</f>
         <v>2462.03125</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="J57">
+        <v>30</v>
+      </c>
+      <c r="K57">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" s="18">
         <v>2</v>
       </c>
@@ -6138,7 +7721,7 @@
         <v>2501.58203125</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" s="18">
         <v>3</v>
       </c>
@@ -6171,7 +7754,7 @@
         <v>2541.8743896484366</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="18">
         <v>4</v>
       </c>
@@ -6204,7 +7787,7 @@
         <v>2582.920684814454</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" s="18">
         <v>5</v>
       </c>
@@ -6237,7 +7820,7 @@
         <v>2624.7334694862348</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" s="18">
         <v>6</v>
       </c>
@@ -6270,7 +7853,7 @@
         <v>2667.3254924178127</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" s="18">
         <v>7</v>
       </c>
@@ -6303,7 +7886,7 @@
         <v>2710.7097013180683</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" s="18">
         <v>8</v>
       </c>

</xml_diff>